<commit_message>
Fill bug registry with fix results
Заполнены колонки N, Q, S, T, Y листа «Реестр багов» по итогам исправлений (коммит b6fe6bc): статусы, дата фикса, коммит, что исправлено, комментарии. Правка выполнена в XML книги, формулы (A, R, X), проверки данных и вложенные объекты сохранены.
</commit_message>
<xml_diff>
--- a/Bug-Tracker-WebPlant.xlsx
+++ b/Bug-Tracker-WebPlant.xlsx
@@ -11,7 +11,7 @@
   <definedNames>
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Реестр багов'!$A$1:$Y$292</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -2487,8 +2487,10 @@
       <c r="M2" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="N2" s="16" t="s">
-        <v>22</v>
+      <c r="N2" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O2" s="15" t="s">
         <v>63</v>
@@ -2496,13 +2498,23 @@
       <c r="P2" s="17">
         <v>46303.0</v>
       </c>
-      <c r="Q2" s="13"/>
+      <c r="Q2" s="13">
+        <v>46305</v>
+      </c>
       <c r="R2" s="18" t="str">
         <f t="shared" ref="R2:R292" si="1">IF(AND($B2&lt;&gt;"",$Q2&lt;&gt;""),$Q2-$B2,"")</f>
         <v/>
       </c>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
+      <c r="S2" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T2" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Тёмная тема: белая карточка шага 2 «Частота полива» и соседние светлые поверхности не перекрашивались. Добавлены правила в addPlants/dark-theme.css для .wateringFrequency, .wateringPreset, .customSchedule, .askAI, .wateringWeekday.</t>
+        </is>
+      </c>
       <c r="U2" s="14"/>
       <c r="V2" s="13"/>
       <c r="W2" s="14"/>
@@ -2510,7 +2522,11 @@
         <f t="shared" ref="X2:X292" si="2">IF(AND($P2&lt;&gt;"",$Q2="",$P2&lt;TODAY(),OR($N2="Новый",$N2="В работе",$N2="На проверке (QA)",$N2="Отложен")),"ДА","")</f>
         <v>ДА</v>
       </c>
-      <c r="Y2" s="12"/>
+      <c r="Y2" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на iPhone в тёмной теме: шаг 2 «Частота полива».</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="str">
@@ -2763,8 +2779,10 @@
       <c r="M6" s="15" t="s">
         <v>246</v>
       </c>
-      <c r="N6" s="25" t="s">
-        <v>22</v>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O6" s="24" t="s">
         <v>63</v>
@@ -2772,13 +2790,23 @@
       <c r="P6" s="17">
         <v>46303.0</v>
       </c>
-      <c r="Q6" s="29"/>
+      <c r="Q6" s="29">
+        <v>46305</v>
+      </c>
       <c r="R6" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
+      <c r="S6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Плашка «Настройки cookie» показывалась на всех страницах, кроме /home, и после согласия читалась как неисчезнувшее уведомление. Теперь она не выводится на /login и /register, где согласия вынесены в саму форму.</t>
+        </is>
+      </c>
       <c r="U6" s="28"/>
       <c r="V6" s="29"/>
       <c r="W6" s="28"/>
@@ -2786,7 +2814,11 @@
         <f t="shared" si="2"/>
         <v>ДА</v>
       </c>
-      <c r="Y6" s="22"/>
+      <c r="Y6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проверить: согласиться с cookie на /login — уведомление и плашка исчезают.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="str">
@@ -2969,8 +3001,10 @@
       <c r="M9" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="N9" s="16" t="s">
-        <v>22</v>
+      <c r="N9" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O9" s="15" t="s">
         <v>63</v>
@@ -2978,13 +3012,23 @@
       <c r="P9" s="17">
         <v>46303.0</v>
       </c>
-      <c r="Q9" s="13"/>
+      <c r="Q9" s="13">
+        <v>46305</v>
+      </c>
       <c r="R9" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
+      <c r="S9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Диалог ИИ-подсказки (.wateringAdviceDialog) оставался светлым в тёмной теме: перекрашены оболочка диалога, шапка, кнопка закрытия и подписи.</t>
+        </is>
+      </c>
       <c r="U9" s="14"/>
       <c r="V9" s="13"/>
       <c r="W9" s="14"/>
@@ -2992,7 +3036,11 @@
         <f t="shared" si="2"/>
         <v>ДА</v>
       </c>
-      <c r="Y9" s="12"/>
+      <c r="Y9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на iPhone в тёмной теме: шаг 2 → «Спросить ИИ».</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="30" t="str">
@@ -3040,7 +3088,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y10" s="30"/>
+      <c r="Y10" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужны уточнения: в отчёте не заполнены шаги воспроизведения, ожидаемый и фактический результат, серьёзность, приоритет и окружение. Без них баг не воспроизводится — добавьте, пожалуйста, шаги, экран/разрешение и скриншот.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="str">
@@ -3083,8 +3135,10 @@
       <c r="M11" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="N11" s="16" t="s">
-        <v>55</v>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Исправлен</t>
+        </is>
       </c>
       <c r="O11" s="15" t="s">
         <v>63</v>
@@ -3093,16 +3147,22 @@
         <v>46305.0</v>
       </c>
       <c r="Q11" s="21">
-        <v>46304.0</v>
+        <v>46305</v>
       </c>
       <c r="R11" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="S11" s="15" t="s">
-        <v>247</v>
-      </c>
-      <c r="T11" s="12"/>
+      <c r="S11" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Причина: просроченная позиция расписания одновременно считалась плановой. Теперь прошедшие позиции расписания не попадают в план (partitionScheduleDates), у дня одна согласованная отметка (resolveWateringMarkers), просрочка считается до первого полива после слота.</t>
+        </is>
+      </c>
       <c r="U11" s="14"/>
       <c r="V11" s="13"/>
       <c r="W11" s="14"/>
@@ -3110,7 +3170,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y11" s="12"/>
+      <c r="Y11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Повторное закрытие: коммит b92f5e7 причину не устранил. Покрыто юнит-тестами (Frontend/src/utils/date.test.js, Backend/utils/wateringSchedule.test.js).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="str">
@@ -3153,8 +3217,10 @@
       <c r="M12" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="N12" s="25" t="s">
-        <v>55</v>
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Исправлен</t>
+        </is>
       </c>
       <c r="O12" s="15" t="s">
         <v>63</v>
@@ -3163,16 +3229,22 @@
         <v>46305.0</v>
       </c>
       <c r="Q12" s="21">
-        <v>46304.0</v>
+        <v>46305</v>
       </c>
       <c r="R12" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="S12" s="15" t="s">
-        <v>247</v>
-      </c>
-      <c r="T12" s="22"/>
+      <c r="S12" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T12" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Просроченный полив больше не «пропадает»: дата остаётся помеченной как пропущенная, карточка дня открывается с событием «Просрочено/Пропущено», а просрочка не застревает на «1 день» — считается до текущего момента либо до первого полива после слота.</t>
+        </is>
+      </c>
       <c r="U12" s="28"/>
       <c r="V12" s="29"/>
       <c r="W12" s="28"/>
@@ -3180,7 +3252,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y12" s="22"/>
+      <c r="Y12" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Повторное закрытие: коммит b92f5e7 причину не устранил. Проверено на сценарии из отчёта (интервал 2 дня, пропуски 7 и 9 октября).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="str">
@@ -3223,8 +3299,10 @@
       <c r="M13" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="N13" s="16" t="s">
-        <v>22</v>
+      <c r="N13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O13" s="15" t="s">
         <v>63</v>
@@ -3232,13 +3310,23 @@
       <c r="P13" s="17">
         <v>46305.0</v>
       </c>
-      <c r="Q13" s="13"/>
+      <c r="Q13" s="13">
+        <v>46305</v>
+      </c>
       <c r="R13" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S13" s="12"/>
-      <c r="T13" s="12"/>
+      <c r="S13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На странице профиля секция «Мои растения» была пустой: заголовок и ссылка «Все» без списка. Пустой блок убран, список растений доступен в разделе «Мои растения».</t>
+        </is>
+      </c>
       <c r="U13" s="14"/>
       <c r="V13" s="13"/>
       <c r="W13" s="14"/>
@@ -3246,7 +3334,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y13" s="12"/>
+      <c r="Y13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на WEB, Chrome, full hd.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="22" t="str">
@@ -3289,8 +3381,10 @@
       <c r="M14" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="N14" s="16" t="s">
-        <v>22</v>
+      <c r="N14" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O14" s="15" t="s">
         <v>63</v>
@@ -3298,13 +3392,23 @@
       <c r="P14" s="17">
         <v>46305.0</v>
       </c>
-      <c r="Q14" s="29"/>
+      <c r="Q14" s="29">
+        <v>46305</v>
+      </c>
       <c r="R14" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S14" s="22"/>
-      <c r="T14" s="22"/>
+      <c r="S14" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T14" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вёрстка «ехала» из-за отступов в процентах от ширины окна (margin 10%/5%, padding 3%): проценты заменены на px, контент ограничен 480px и центрирован, форма больше не растягивается на широком экране.</t>
+        </is>
+      </c>
       <c r="U14" s="28"/>
       <c r="V14" s="29"/>
       <c r="W14" s="28"/>
@@ -3312,7 +3416,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y14" s="22"/>
+      <c r="Y14" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на WEB 1920×1080.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="str">
@@ -3355,8 +3463,10 @@
       <c r="M15" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="N15" s="16" t="s">
-        <v>22</v>
+      <c r="N15" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O15" s="15" t="s">
         <v>63</v>
@@ -3364,13 +3474,23 @@
       <c r="P15" s="17">
         <v>46305.0</v>
       </c>
-      <c r="Q15" s="13"/>
+      <c r="Q15" s="13">
+        <v>46305</v>
+      </c>
       <c r="R15" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S15" s="12"/>
-      <c r="T15" s="12"/>
+      <c r="S15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Верхний блок с кнопкой «Назад» уходил под чёлку: в отступы страницы добавлен env(safe-area-inset-*), включая мобильные media-запросы.</t>
+        </is>
+      </c>
       <c r="U15" s="14"/>
       <c r="V15" s="13"/>
       <c r="W15" s="14"/>
@@ -3378,7 +3498,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y15" s="12"/>
+      <c r="Y15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на iPhone, в том числе в установленном PWA.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="22" t="str">
@@ -3561,8 +3685,10 @@
       <c r="M18" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="N18" s="25" t="s">
-        <v>22</v>
+      <c r="N18" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O18" s="24" t="s">
         <v>63</v>
@@ -3570,13 +3696,23 @@
       <c r="P18" s="23">
         <v>46306.0</v>
       </c>
-      <c r="Q18" s="29"/>
+      <c r="Q18" s="29">
+        <v>46305</v>
+      </c>
       <c r="R18" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S18" s="22"/>
-      <c r="T18" s="22"/>
+      <c r="S18" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T18" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">В альбомной ориентации календарь растягивался на всю ширину и не приходил в норму после возврата в портретную. Добавлен ландшафтный режим: мобильная колонка держится шириной до 520px по центру. Блокировка поворота уже запрошена в манифесте (orientation: portrait-primary), но iOS её игнорирует, поэтому нужен именно устойчивый ландшафтный layout.</t>
+        </is>
+      </c>
       <c r="U18" s="28"/>
       <c r="V18" s="29"/>
       <c r="W18" s="28"/>
@@ -3584,7 +3720,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y18" s="22"/>
+      <c r="Y18" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на iPhone: повернуть в альбомную ориентацию и обратно.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="str">
@@ -3627,8 +3767,10 @@
       <c r="M19" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="N19" s="16" t="s">
-        <v>22</v>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На проверке (QA)</t>
+        </is>
       </c>
       <c r="O19" s="24" t="s">
         <v>63</v>
@@ -3636,13 +3778,23 @@
       <c r="P19" s="23">
         <v>46306.0</v>
       </c>
-      <c r="Q19" s="13"/>
+      <c r="Q19" s="13">
+        <v>46305</v>
+      </c>
       <c r="R19" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S19" s="12"/>
-      <c r="T19" s="12"/>
+      <c r="S19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Причина: у .screenTransition стоял will-change: transform, из-за чего он становился containing block для position: fixed — модалка дня позиционировалась от прокручиваемого блока (уезжала при скролле), а нижнее меню рисовалось поверх оверлея. Модалка перенесена в портал к body, will-change заменён на opacity, прокрутка фона блокируется через body.vision-open.</t>
+        </is>
+      </c>
       <c r="U19" s="14"/>
       <c r="V19" s="13"/>
       <c r="W19" s="14"/>
@@ -3650,7 +3802,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y19" s="12"/>
+      <c r="Y19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужна проверка на iPhone: открыть день с поливом, прокрутить, посмотреть на нижнее меню.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="22" t="str">
@@ -3693,8 +3849,10 @@
       <c r="M20" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="N20" s="25" t="s">
-        <v>22</v>
+      <c r="N20" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Исправлен</t>
+        </is>
       </c>
       <c r="O20" s="24" t="s">
         <v>63</v>
@@ -3702,13 +3860,23 @@
       <c r="P20" s="23">
         <v>46306.0</v>
       </c>
-      <c r="Q20" s="29"/>
+      <c r="Q20" s="29">
+        <v>46305</v>
+      </c>
       <c r="R20" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="S20" s="22"/>
-      <c r="T20" s="22"/>
+      <c r="S20" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6fe6bc</t>
+        </is>
+      </c>
+      <c r="T20" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дни недели подсвечивались все сразу, если частота полива не кратна неделе. Теперь: 7 и 14 дней → конкретный день недели первого полива, «каждый день» → все дни, смещающийся график (3, 4, 10 дней) → ограничение по дням не накладывается, в интерфейсе появилось пояснение.</t>
+        </is>
+      </c>
       <c r="U20" s="28"/>
       <c r="V20" s="29"/>
       <c r="W20" s="28"/>
@@ -3716,7 +3884,11 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Y20" s="22"/>
+      <c r="Y20" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проверено юнит-тестами: Frontend/src/utils/date.test.js (reminderWeekdaysForInterval), 9 тестов — все проходят.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="str">

</xml_diff>